<commit_message>
data(jpg): replace groups 1 and 3 with error-selected receipts
</commit_message>
<xml_diff>
--- a/jpg-ocr-stat/evaluation/group_01/stat_oracle.xlsx
+++ b/jpg-ocr-stat/evaluation/group_01/stat_oracle.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="results" sheetId="1" r:id="R1ba993b0b4aa44a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="results" sheetId="1" r:id="Ra868254bea3c41a8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -276,222 +276,222 @@
     </x:row>
     <x:row r="2" ht="20" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>X51005447839.png</x:v>
+        <x:v>receipt_0011.png</x:v>
       </x:c>
       <x:c r="B2" s="2" t="str">
-        <x:v>2018-03-09</x:v>
+        <x:v>2018-03-12</x:v>
       </x:c>
       <x:c r="C2" s="2" t="str">
-        <x:v>65.20</x:v>
+        <x:v>343.95</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="20" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>X51005447841.png</x:v>
+        <x:v>receipt_0012.png</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
-        <x:v>2018-03-09</x:v>
+        <x:v>2018-02-05</x:v>
       </x:c>
       <x:c r="C3" s="2" t="str">
-        <x:v>10.40</x:v>
+        <x:v>63.60</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="20" customHeight="1">
       <x:c r="A4" s="2" t="str">
-        <x:v>X51005447851.png</x:v>
+        <x:v>receipt_0013.png</x:v>
       </x:c>
       <x:c r="B4" s="2" t="str">
-        <x:v>2018-01-30</x:v>
+        <x:v>2018-03-13</x:v>
       </x:c>
       <x:c r="C4" s="2" t="str">
-        <x:v>1.70</x:v>
+        <x:v>100.90</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
       <x:c r="A5" s="2" t="str">
-        <x:v>X51005568866.png</x:v>
+        <x:v>receipt_0014.png</x:v>
       </x:c>
       <x:c r="B5" s="2" t="str">
-        <x:v>2017-08-20</x:v>
+        <x:v>2018-02-06</x:v>
       </x:c>
       <x:c r="C5" s="2" t="str">
-        <x:v>5.05</x:v>
+        <x:v>14.65</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
       <x:c r="A6" s="2" t="str">
-        <x:v>X51005568880.png</x:v>
+        <x:v>receipt_0018.png</x:v>
       </x:c>
       <x:c r="B6" s="2" t="str">
-        <x:v>2017-09-19</x:v>
+        <x:v>2018-02-06</x:v>
       </x:c>
       <x:c r="C6" s="2" t="str">
-        <x:v>15.90</x:v>
+        <x:v>109.70</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
       <x:c r="A7" s="2" t="str">
-        <x:v>X51005568889.png</x:v>
+        <x:v>receipt_0031.png</x:v>
       </x:c>
       <x:c r="B7" s="2" t="str">
-        <x:v>2017-02-11</x:v>
+        <x:v>2018-01-13</x:v>
       </x:c>
       <x:c r="C7" s="2" t="str">
-        <x:v>19.60</x:v>
+        <x:v>6.36</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
       <x:c r="A8" s="2" t="str">
-        <x:v>X51005568899.png</x:v>
+        <x:v>receipt_0053.png</x:v>
       </x:c>
       <x:c r="B8" s="2" t="str">
-        <x:v>2017-10-18</x:v>
+        <x:v>2018-02-28</x:v>
       </x:c>
       <x:c r="C8" s="2" t="str">
-        <x:v>5.90</x:v>
+        <x:v>10.45</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="20" customHeight="1">
       <x:c r="A9" s="2" t="str">
-        <x:v>X51005587267.png</x:v>
+        <x:v>receipt_0059.png</x:v>
       </x:c>
       <x:c r="B9" s="2" t="str">
-        <x:v>2017-02-04</x:v>
+        <x:v>2017-04-23</x:v>
       </x:c>
       <x:c r="C9" s="2" t="str">
-        <x:v>85.10</x:v>
+        <x:v>12.35</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="20" customHeight="1">
       <x:c r="A10" s="2" t="str">
-        <x:v>X51005675103.png</x:v>
+        <x:v>receipt_0068.png</x:v>
       </x:c>
       <x:c r="B10" s="2" t="str">
-        <x:v>2018-01-04</x:v>
+        <x:v>2018-04-13</x:v>
       </x:c>
       <x:c r="C10" s="2" t="str">
-        <x:v>100.17</x:v>
+        <x:v>27.00</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="20" customHeight="1">
       <x:c r="A11" s="2" t="str">
-        <x:v>X51005676536.png</x:v>
+        <x:v>receipt_0080.png</x:v>
       </x:c>
       <x:c r="B11" s="2" t="str">
-        <x:v>2018-01-02</x:v>
+        <x:v>2018-05-13</x:v>
       </x:c>
       <x:c r="C11" s="2" t="str">
-        <x:v>93.07</x:v>
+        <x:v>22.90</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20" customHeight="1">
       <x:c r="A12" s="2" t="str">
-        <x:v>X51005676540.png</x:v>
+        <x:v>receipt_0081.png</x:v>
       </x:c>
       <x:c r="B12" s="2" t="str">
-        <x:v>2018-01-11</x:v>
+        <x:v>2018-02-12</x:v>
       </x:c>
       <x:c r="C12" s="2" t="str">
-        <x:v>116.28</x:v>
+        <x:v>112.45</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="20" customHeight="1">
       <x:c r="A13" s="2" t="str">
-        <x:v>X51005676546.png</x:v>
+        <x:v>receipt_0082.png</x:v>
       </x:c>
       <x:c r="B13" s="2" t="str">
-        <x:v>2018-01-11</x:v>
+        <x:v>2018-02-16</x:v>
       </x:c>
       <x:c r="C13" s="2" t="str">
-        <x:v>21.20</x:v>
+        <x:v>21.50</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="20" customHeight="1">
       <x:c r="A14" s="2" t="str">
-        <x:v>X51005677331.png</x:v>
+        <x:v>receipt_0088.png</x:v>
       </x:c>
       <x:c r="B14" s="2" t="str">
-        <x:v>2018-02-03</x:v>
+        <x:v>2018-04-06</x:v>
       </x:c>
       <x:c r="C14" s="2" t="str">
-        <x:v>60.95</x:v>
+        <x:v>270.00</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="20" customHeight="1">
       <x:c r="A15" s="2" t="str">
-        <x:v>X51005705727.png</x:v>
+        <x:v>receipt_0107.png</x:v>
       </x:c>
       <x:c r="B15" s="2" t="str">
-        <x:v>2017-12-28</x:v>
+        <x:v>2018-02-12</x:v>
       </x:c>
       <x:c r="C15" s="2" t="str">
-        <x:v>38.15</x:v>
+        <x:v>5.30</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="20" customHeight="1">
       <x:c r="A16" s="2" t="str">
-        <x:v>X51005705729.png</x:v>
+        <x:v>receipt_0113.png</x:v>
       </x:c>
       <x:c r="B16" s="2" t="str">
-        <x:v>2017-10-13</x:v>
+        <x:v>2018-02-01</x:v>
       </x:c>
       <x:c r="C16" s="2" t="str">
-        <x:v>94.60</x:v>
+        <x:v>20.50</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="20" customHeight="1">
       <x:c r="A17" s="2" t="str">
-        <x:v>X51005711453.png</x:v>
+        <x:v>receipt_0114.png</x:v>
       </x:c>
       <x:c r="B17" s="2" t="str">
-        <x:v>2018-03-10</x:v>
+        <x:v>2018-02-02</x:v>
       </x:c>
       <x:c r="C17" s="2" t="str">
-        <x:v>8.50</x:v>
+        <x:v>48.00</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="20" customHeight="1">
       <x:c r="A18" s="2" t="str">
-        <x:v>X51005719855.png</x:v>
+        <x:v>receipt_0149.png</x:v>
       </x:c>
       <x:c r="B18" s="2" t="str">
-        <x:v>2018-02-19</x:v>
+        <x:v>2017-01-05</x:v>
       </x:c>
       <x:c r="C18" s="2" t="str">
-        <x:v>181.55</x:v>
+        <x:v>12.60</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="20" customHeight="1">
       <x:c r="A19" s="2" t="str">
-        <x:v>X51005719857.png</x:v>
+        <x:v>receipt_0181.png</x:v>
       </x:c>
       <x:c r="B19" s="2" t="str">
-        <x:v>2018-02-19</x:v>
+        <x:v>2018-03-28</x:v>
       </x:c>
       <x:c r="C19" s="2" t="str">
-        <x:v>23.80</x:v>
+        <x:v>30.00</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="20" customHeight="1">
       <x:c r="A20" s="2" t="str">
-        <x:v>X51005719895.png</x:v>
+        <x:v>receipt_0184.png</x:v>
       </x:c>
       <x:c r="B20" s="2" t="str">
-        <x:v>2018-08-01</x:v>
+        <x:v>2018-03-12</x:v>
       </x:c>
       <x:c r="C20" s="2" t="str">
-        <x:v>34.80</x:v>
+        <x:v>42.50</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="20" customHeight="1">
       <x:c r="A21" s="2" t="str">
-        <x:v>X51005724629.png</x:v>
+        <x:v>receipt_0185.png</x:v>
       </x:c>
       <x:c r="B21" s="2" t="str">
-        <x:v>2018-03-17</x:v>
+        <x:v>2018-03-29</x:v>
       </x:c>
       <x:c r="C21" s="2" t="str">
-        <x:v>174.90</x:v>
+        <x:v>100.60</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>